<commit_message>
done xlsx product name
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/qSHProductImportSchema_en.xlsx
+++ b/src/main/resources/qm/public/resources/qSHProductImportSchema_en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qcadoo_demo_clone\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675F2145-5855-4F89-A5EE-49CEFC8BD7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2644D716-CC0D-48A2-8433-9167A10FF7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C3DD0E6-ED60-435A-92B4-4D6BBCAE0B6F}"/>
+    <workbookView xWindow="6300" yWindow="4080" windowWidth="21600" windowHeight="11235" xr2:uid="{1C3DD0E6-ED60-435A-92B4-4D6BBCAE0B6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>Product number</t>
+  </si>
+  <si>
+    <t>Product name</t>
   </si>
 </sst>
 </file>
@@ -421,15 +424,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6EA1A54-C7AA-4FC5-B4D4-E1F04F5DAE96}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>